<commit_message>
Instruction atten added, bug fixed
</commit_message>
<xml_diff>
--- a/tables/AttenuatorDiconPassport.xlsx
+++ b/tables/AttenuatorDiconPassport.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23001"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5144C3E0-7546-462B-B9DE-2F4DE79FC5BA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3384844F-5900-4B98-B47B-0404D51651E5}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-13080" yWindow="1785" windowWidth="14400" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <t>Voltage (V)</t>
   </si>
   <si>
-    <t>Attenuation (dBm)</t>
+    <t>Attenuation (dB)</t>
   </si>
 </sst>
 </file>

</xml_diff>